<commit_message>
Initialized PortScan script, wait for Mark response
</commit_message>
<xml_diff>
--- a/MultiProgram/stats_bb_noper_16/Data Comparison.xlsx
+++ b/MultiProgram/stats_bb_noper_16/Data Comparison.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexb\OneDrive\Documents\Thesis\MultiProgram\stats_bb_noper_16\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{D6803797-7BE0-498C-B304-724EF27C4669}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A78CEFB-AD99-4D20-95CC-817561A706BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3760" yWindow="3760" windowWidth="28800" windowHeight="15910" xr2:uid="{D88461B2-2C65-4402-BC28-F6BD8FEB8E0C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{D88461B2-2C65-4402-BC28-F6BD8FEB8E0C}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Comparison" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -4829,7 +4842,7 @@
         <v>8</v>
       </c>
       <c r="AZ37">
-        <f t="shared" ref="AZ37:AZ52" si="1">AS37-AL37</f>
+        <f t="shared" ref="AZ37:AZ51" si="1">AS37-AL37</f>
         <v>11014853</v>
       </c>
       <c r="BA37">

</xml_diff>